<commit_message>
Update 664204 - MSCI ACWI IMI Index .xlsx
</commit_message>
<xml_diff>
--- a/data/664204 - MSCI ACWI IMI Index .xlsx
+++ b/data/664204 - MSCI ACWI IMI Index .xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7629" uniqueCount="7628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7652" uniqueCount="7651">
   <si>
     <t>Index Level:</t>
   </si>
@@ -22895,6 +22895,75 @@
   </si>
   <si>
     <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -23280,7 +23349,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E7613"/>
+  <dimension ref="A3:E7636"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -84221,6 +84290,190 @@
         <v>3432.089938</v>
       </c>
     </row>
+    <row r="7614" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7614" t="s">
+        <v>7628</v>
+      </c>
+      <c r="B7614">
+        <v>3496.286178</v>
+      </c>
+    </row>
+    <row r="7615" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7615" t="s">
+        <v>7629</v>
+      </c>
+      <c r="B7615">
+        <v>3561.010848</v>
+      </c>
+    </row>
+    <row r="7616" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7616" t="s">
+        <v>7630</v>
+      </c>
+      <c r="B7616">
+        <v>3548.504616</v>
+      </c>
+    </row>
+    <row r="7617" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7617" t="s">
+        <v>7631</v>
+      </c>
+      <c r="B7617">
+        <v>3552.527773</v>
+      </c>
+    </row>
+    <row r="7618" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7618" t="s">
+        <v>7632</v>
+      </c>
+      <c r="B7618">
+        <v>3564.965292</v>
+      </c>
+    </row>
+    <row r="7619" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7619" t="s">
+        <v>7633</v>
+      </c>
+      <c r="B7619">
+        <v>3566.609078</v>
+      </c>
+    </row>
+    <row r="7620" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7620" t="s">
+        <v>7634</v>
+      </c>
+      <c r="B7620">
+        <v>3685.847387</v>
+      </c>
+    </row>
+    <row r="7621" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7621" t="s">
+        <v>7635</v>
+      </c>
+      <c r="B7621">
+        <v>3691.363248</v>
+      </c>
+    </row>
+    <row r="7622" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7622" t="s">
+        <v>7636</v>
+      </c>
+      <c r="B7622">
+        <v>3699.540943</v>
+      </c>
+    </row>
+    <row r="7623" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7623" t="s">
+        <v>7637</v>
+      </c>
+      <c r="B7623">
+        <v>3718.518813</v>
+      </c>
+    </row>
+    <row r="7624" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7624" t="s">
+        <v>7638</v>
+      </c>
+      <c r="B7624">
+        <v>3768.963411</v>
+      </c>
+    </row>
+    <row r="7625" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7625" t="s">
+        <v>7639</v>
+      </c>
+      <c r="B7625">
+        <v>3789.761816</v>
+      </c>
+    </row>
+    <row r="7626" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7626" t="s">
+        <v>7640</v>
+      </c>
+      <c r="B7626">
+        <v>3802.203404</v>
+      </c>
+    </row>
+    <row r="7627" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7627" t="s">
+        <v>7641</v>
+      </c>
+      <c r="B7627">
+        <v>3842.502503</v>
+      </c>
+    </row>
+    <row r="7628" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7628" t="s">
+        <v>7642</v>
+      </c>
+      <c r="B7628">
+        <v>3834.105291</v>
+      </c>
+    </row>
+    <row r="7629" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7629" t="s">
+        <v>7643</v>
+      </c>
+      <c r="B7629">
+        <v>3814.668416</v>
+      </c>
+    </row>
+    <row r="7630" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7630" t="s">
+        <v>7644</v>
+      </c>
+      <c r="B7630">
+        <v>3830.315809</v>
+      </c>
+    </row>
+    <row r="7631" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7631" t="s">
+        <v>7645</v>
+      </c>
+      <c r="B7631">
+        <v>3815.267157</v>
+      </c>
+    </row>
+    <row r="7632" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7632" t="s">
+        <v>7646</v>
+      </c>
+      <c r="B7632">
+        <v>3831.157139</v>
+      </c>
+    </row>
+    <row r="7633" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7633" t="s">
+        <v>7647</v>
+      </c>
+      <c r="B7633">
+        <v>3841.543742</v>
+      </c>
+    </row>
+    <row r="7634" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7634" t="s">
+        <v>7648</v>
+      </c>
+      <c r="B7634">
+        <v>3819.832301</v>
+      </c>
+    </row>
+    <row r="7635" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7635" t="s">
+        <v>7649</v>
+      </c>
+      <c r="B7635">
+        <v>3813.70278</v>
+      </c>
+    </row>
+    <row r="7636" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7636" t="s">
+        <v>7650</v>
+      </c>
+      <c r="B7636">
+        <v>3850.085626</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>